<commit_message>
Addressed issues with the check logic and added an additional postitive test case.
</commit_message>
<xml_diff>
--- a/rules/CORE-001078/positive/01/data/unit-test-coreid-FB0609-positive.xlsx
+++ b/rules/CORE-001078/positive/01/data/unit-test-coreid-FB0609-positive.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -185,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -211,7 +210,7 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -226,7 +225,7 @@
     <xf numFmtId="49" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -286,6 +285,12 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1283,7 +1288,7 @@
       <c r="M5" s="8" t="n">
         <v>701</v>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="N5" s="40" t="n">
         <v>17372</v>
       </c>
       <c r="O5" s="7" t="inlineStr">
@@ -1401,7 +1406,7 @@
       <c r="M6" s="14" t="n">
         <v>701</v>
       </c>
-      <c r="N6" s="16" t="n">
+      <c r="N6" s="41" t="n">
         <v>1955</v>
       </c>
       <c r="O6" s="12" t="inlineStr">
@@ -1519,7 +1524,7 @@
       <c r="M7" s="8" t="n">
         <v>701</v>
       </c>
-      <c r="N7" s="11" t="n">
+      <c r="N7" s="40" t="n">
         <v>16239</v>
       </c>
       <c r="O7" s="7" t="inlineStr">
@@ -1629,7 +1634,7 @@
       <c r="M8" s="8" t="n">
         <v>701</v>
       </c>
-      <c r="N8" s="11" t="n">
+      <c r="N8" s="40" t="n">
         <v>1933</v>
       </c>
       <c r="O8" s="7" t="inlineStr">
@@ -1747,7 +1752,7 @@
       <c r="M9" s="8" t="n">
         <v>701</v>
       </c>
-      <c r="N9" s="16" t="n">
+      <c r="N9" s="41" t="n">
         <v>1955</v>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -2114,7 +2119,11 @@
           <t>FATAL</t>
         </is>
       </c>
-      <c r="G7" s="30" t="n"/>
+      <c r="G7" s="30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H7" s="29" t="inlineStr">
         <is>
           <t>2018-08-14</t>
@@ -2238,7 +2247,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F10" s="30" t="n"/>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>FATAL</t>
+        </is>
+      </c>
       <c r="G10" s="30" t="inlineStr">
         <is>
           <t>Y</t>

</xml_diff>